<commit_message>
Confirm velocity limits against real Jordanian code, flag slope basis conflict
Added the Jordanian plumbing code (Codes/plumbing_Code.pdf) and checked it
against the three Phase 2 reference tables flagged as not independently
Jordan-confirmed (SOP §5a). Domestic water velocity is now resolved:
VelocityLimits.xlsx cold-water max updated 2.4->2.5 m/s to match the
code's explicit text; hot-water row already matched and is now cited
directly. Drainage minimum slope surfaced a real basis conflict (the
code's flat 2%/1% UPC-style rule vs. the table's IPC-704.1 diameter-tiered
values) - logged in PROCEDURE.md §24 for senior review rather than applied
unilaterally, since it would change FAIL counts firm-wide.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel_templates/VelocityLimits.xlsx
+++ b/docs/excel_templates/VelocityLimits.xlsx
@@ -612,16 +612,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ASPE Data Book / IPC</t>
+          <t>Jordanian National Building Code - Unified Plumbing Code (2013) Section 6.10.12 / ASPE Data Book</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8 ft/s (2.4 m/s) max is the commonly cited ceiling for copper cold-water piping to limit erosion; matches IPC guidance.</t>
+          <t>Jordanian code Section 6.10.12 states max 2.5 m/s for cold water in copper pipe/fittings and in non-copper pipe using copper-alloy fittings (matches UPC-derived national code text, Codes/plumbing_Code.pdf). Supersedes the prior 2.4 m/s (8 ft/s) ASPE/IPC-sourced ceiling.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -646,12 +646,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ASPE Data Book / IPC</t>
+          <t>Jordanian National Building Code - Unified Plumbing Code (2013) Section 6.10.12 / ASPE Data Book</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>5 ft/s (1.5 m/s) max for hot water — lower than cold water because erosion-corrosion accelerates with temperature.</t>
+          <t>Jordanian code Section 6.10.12 confirms max 1.5 m/s for hot water in copper pipe/fittings and in non-copper pipe using copper-alloy fittings -- matches the prior ASPE/IPC-sourced value exactly (Codes/plumbing_Code.pdf).</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>